<commit_message>
fix(wallet-batch): update expiry batch file [EGCMS-1079] (#15571)
* fix(wallet-batch): update expiry batch file

* update file

* uncomment checks
</commit_message>
<xml_diff>
--- a/public/files/sample_extend_gift_card_expiry.xlsx
+++ b/public/files/sample_extend_gift_card_expiry.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="Batch test mayank - Sheet1" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -22,6 +22,12 @@
     <t>Expiry (YYYY-MM-DD)</t>
   </si>
   <si>
+    <t>Reference ID (Optional)</t>
+  </si>
+  <si>
+    <t>Notes (Optional)</t>
+  </si>
+  <si>
     <t>Contact</t>
   </si>
   <si>
@@ -32,19 +38,13 @@
   </si>
   <si>
     <t>Source</t>
-  </si>
-  <si>
-    <t>Reference ID (Optional)</t>
-  </si>
-  <si>
-    <t>Notes (Optional)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -52,62 +52,31 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border/>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -322,10 +291,14 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="25.75"/>
-    <col customWidth="1" min="3" max="7" width="19.5"/>
-    <col customWidth="1" min="8" max="8" width="22.88"/>
-    <col customWidth="1" min="9" max="9" width="15.5"/>
+    <col customWidth="1" min="1" max="1" width="20.88"/>
+    <col customWidth="1" min="2" max="2" width="26.63"/>
+    <col customWidth="1" min="3" max="3" width="27.25"/>
+    <col customWidth="1" min="4" max="4" width="18.0"/>
+    <col customWidth="1" min="5" max="5" width="18.38"/>
+    <col customWidth="1" min="6" max="6" width="14.5"/>
+    <col customWidth="1" min="8" max="8" width="15.88"/>
+    <col customWidth="1" min="9" max="9" width="13.88"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -350,10 +323,10 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>